<commit_message>
Refactor dashboard and align master table export
</commit_message>
<xml_diff>
--- a/templates/Template Tabla Maestra.xlsx
+++ b/templates/Template Tabla Maestra.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanPedro\Desktop\WorkSpace\followup\audit-automation\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C3F74F6-48EE-4C8D-8286-CB5C67AA7D81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FA4DE6A-417F-4F60-B2E8-8AFAE7093466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>Datos base</t>
   </si>
@@ -125,6 +125,9 @@
   </si>
   <si>
     <t>% Precision de Género</t>
+  </si>
+  <si>
+    <t>Tipo_sensor</t>
   </si>
 </sst>
 </file>
@@ -584,16 +587,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -612,6 +609,9 @@
         </ext>
       </extLst>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -624,6 +624,9 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -631,198 +634,12 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="61">
+  <dxfs count="63">
     <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center"/>
     </dxf>
     <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF6F8F9"/>
-          <bgColor rgb="FFF6F8F9"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border outline="0">
-        <left/>
-        <right style="thin">
-          <color rgb="FF373F6B"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF6F8F9"/>
-          <bgColor rgb="FFF6F8F9"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border outline="0">
-        <left/>
-        <right style="thin">
-          <color rgb="FF373F6B"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF6F8F9"/>
-          <bgColor rgb="FFF6F8F9"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF6F8F9"/>
-          <bgColor rgb="FFF6F8F9"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF6F8F9"/>
-          <bgColor rgb="FFF6F8F9"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF6F8F9"/>
-          <bgColor rgb="FFF6F8F9"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF6F8F9"/>
-          <bgColor rgb="FFF6F8F9"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center"/>
     </dxf>
     <dxf>
       <font>
@@ -1427,6 +1244,198 @@
       <alignment horizontal="center" vertical="center"/>
     </dxf>
     <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
+        <left/>
+        <right style="thin">
+          <color rgb="FF373F6B"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
+        <left/>
+        <right style="thin">
+          <color rgb="FF373F6B"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center"/>
     </dxf>
     <dxf>
@@ -1589,14 +1598,14 @@
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="TABLA MAESTRA-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="60"/>
-      <tableStyleElement type="headerRow" dxfId="59"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="62"/>
+      <tableStyleElement type="headerRow" dxfId="61"/>
+      <tableStyleElement type="firstRowStripe" dxfId="60"/>
+      <tableStyleElement type="secondRowStripe" dxfId="59"/>
+    </tableStyle>
+    <tableStyle name="TABLA MAESTRA-style 2" pivot="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
       <tableStyleElement type="firstRowStripe" dxfId="58"/>
       <tableStyleElement type="secondRowStripe" dxfId="57"/>
-    </tableStyle>
-    <tableStyle name="TABLA MAESTRA-style 2" pivot="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <tableStyleElement type="firstRowStripe" dxfId="56"/>
-      <tableStyleElement type="secondRowStripe" dxfId="55"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1628,75 +1637,76 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla_1" displayName="Tabla_1" ref="A2:AA11" headerRowDxfId="54" dataDxfId="53" totalsRowDxfId="52">
-  <tableColumns count="27">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Zona" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Fecha" dataDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla_1" displayName="Tabla_1" ref="A2:AB11" headerRowDxfId="56" dataDxfId="55" totalsRowDxfId="54">
+  <tableColumns count="28">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Zona" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Fecha" dataDxfId="52">
       <calculatedColumnFormula>IFERROR(ROUND(INDEX($Q:$Q,ROW())/INDEX($F:$F,ROW())*100,2),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Hora inicio (UTC 0)" dataDxfId="49"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Hora término" dataDxfId="48">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Hora inicio (UTC 0)" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Hora término" dataDxfId="50">
       <calculatedColumnFormula>IFERROR(ROUND(INDEX($Q:$Q,ROW())/INDEX($F:$F,ROW())*100,2),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Cámara" dataDxfId="47"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Total Eventos" dataDxfId="46">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Cámara" dataDxfId="49"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Total Eventos" dataDxfId="48">
       <calculatedColumnFormula>IFERROR(ROUND(INDEX($Q:$Q,ROW())/INDEX($F:$F,ROW())*100,2),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Eventos Registrados por el Sistema" dataDxfId="45"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="% Eventos Registrados por el Sistema" dataDxfId="44">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Eventos Registrados por el Sistema" dataDxfId="47"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="% Eventos Registrados por el Sistema" dataDxfId="46">
       <calculatedColumnFormula>IFERROR(ROUND(INDEX($Q:$Q,ROW())/INDEX($F:$F,ROW())*100,2),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Eventos NO Registrados (Manuales)" dataDxfId="43"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="% Eventos NO Registrados (Manuales)" dataDxfId="42">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Eventos NO Registrados (Manuales)" dataDxfId="45"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="% Eventos NO Registrados (Manuales)" dataDxfId="44">
       <calculatedColumnFormula>IFERROR(ROUND(INDEX($Q:$Q,ROW())/INDEX($F:$F,ROW())*100,2),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Eventos Correctos del Sistema" dataDxfId="41"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="% Eventos Correctos sobre Registrados" dataDxfId="40"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="% Eventos Correctos sobre Total" dataDxfId="39"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Eventos Reg. Mal (Sist.)" dataDxfId="38"/>
-    <tableColumn id="32" xr3:uid="{3DDF4720-C83D-42B1-92F8-BF7BF81CA800}" name="% Eventos Reg. Mal sobre Registrados" dataDxfId="12"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Cobertura Identity" dataDxfId="5"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="% Cobertura Identity" dataDxfId="11"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Identity Unknown" dataDxfId="4"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="% Identity Unknown" dataDxfId="10"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Cobertura Género" dataDxfId="3"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="% Cobertura Género" dataDxfId="9"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Precision de Género" dataDxfId="2"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="% Precision de Género" dataDxfId="8"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Cobertura Edad" dataDxfId="1"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="% Cobertura Edad" dataDxfId="7"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Precisión de Edad" dataDxfId="0"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="% Precisión de Edad" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Eventos Correctos del Sistema" dataDxfId="43"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="% Eventos Correctos sobre Registrados" dataDxfId="42"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="% Eventos Correctos sobre Total" dataDxfId="41"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Eventos Reg. Mal (Sist.)" dataDxfId="40"/>
+    <tableColumn id="32" xr3:uid="{3DDF4720-C83D-42B1-92F8-BF7BF81CA800}" name="% Eventos Reg. Mal sobre Registrados" dataDxfId="39"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Cobertura Identity" dataDxfId="38"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="% Cobertura Identity" dataDxfId="37"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Identity Unknown" dataDxfId="36"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="% Identity Unknown" dataDxfId="35"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Cobertura Género" dataDxfId="34"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="% Cobertura Género" dataDxfId="33"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Precision de Género" dataDxfId="32"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="% Precision de Género" dataDxfId="31"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Cobertura Edad" dataDxfId="30"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="% Cobertura Edad" dataDxfId="29"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Precisión de Edad" dataDxfId="28"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="% Precisión de Edad" dataDxfId="27"/>
+    <tableColumn id="27" xr3:uid="{EE661BE4-91C5-4AE1-84FF-C23068902F9D}" name="Tipo_sensor" dataDxfId="1" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TABLA MAESTRA-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table_1" displayName="Table_1" ref="A13:V13" headerRowCount="0" headerRowDxfId="37" dataDxfId="36" totalsRowDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table_1" displayName="Table_1" ref="A13:V13" headerRowCount="0" headerRowDxfId="26" dataDxfId="25" totalsRowDxfId="24">
   <tableColumns count="22">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Column1" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Column2" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Column3" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Column4" dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Column5" dataDxfId="30"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Column6" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Column7" dataDxfId="28"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Column8" dataDxfId="27"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Column9" dataDxfId="26"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="Column10" dataDxfId="25"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Column11" dataDxfId="24"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Column12" dataDxfId="23"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Column13" dataDxfId="22"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Column14" dataDxfId="21"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="Column15" dataDxfId="20"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Column16" dataDxfId="19"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Column17" dataDxfId="18"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0100-000012000000}" name="Column18" dataDxfId="17"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0100-000013000000}" name="Column19" dataDxfId="16"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0100-000014000000}" name="Column20" dataDxfId="15"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0100-000015000000}" name="Column21" dataDxfId="14"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0100-000016000000}" name="Column22" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Column1" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Column2" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Column3" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Column4" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Column5" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Column6" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Column7" dataDxfId="17"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Column8" dataDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Column9" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="Column10" dataDxfId="14"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Column11" dataDxfId="13"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Column12" dataDxfId="12"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Column13" dataDxfId="11"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Column14" dataDxfId="10"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="Column15" dataDxfId="9"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Column16" dataDxfId="8"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Column17" dataDxfId="7"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0100-000012000000}" name="Column18" dataDxfId="6"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0100-000013000000}" name="Column19" dataDxfId="5"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0100-000014000000}" name="Column20" dataDxfId="4"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0100-000015000000}" name="Column21" dataDxfId="3"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0100-000016000000}" name="Column22" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TABLA MAESTRA-style 2" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1904,7 +1914,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AA995"/>
+  <dimension ref="A1:AB995"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19" style="20" customWidth="1"/>
@@ -1933,14 +1943,14 @@
     <col min="28" max="16384" width="12.5703125" style="20"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="31" t="s">
+    <row r="1" spans="1:28" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="28"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="29"/>
       <c r="F1" s="25" t="s">
         <v>1</v>
       </c>
@@ -1948,33 +1958,33 @@
       <c r="H1" s="26"/>
       <c r="I1" s="26"/>
       <c r="J1" s="27"/>
-      <c r="K1" s="32" t="s">
+      <c r="K1" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="33"/>
-      <c r="M1" s="33"/>
-      <c r="N1" s="33"/>
-      <c r="O1" s="33"/>
-      <c r="P1" s="30" t="s">
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
+      <c r="O1" s="31"/>
+      <c r="P1" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" s="30"/>
-      <c r="R1" s="30"/>
-      <c r="S1" s="34"/>
-      <c r="T1" s="35" t="s">
+      <c r="Q1" s="32"/>
+      <c r="R1" s="32"/>
+      <c r="S1" s="33"/>
+      <c r="T1" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="U1" s="36"/>
-      <c r="V1" s="36"/>
-      <c r="W1" s="37"/>
-      <c r="X1" s="29" t="s">
+      <c r="U1" s="35"/>
+      <c r="V1" s="35"/>
+      <c r="W1" s="36"/>
+      <c r="X1" s="37" t="s">
         <v>5</v>
       </c>
       <c r="Y1" s="38"/>
       <c r="Z1" s="38"/>
       <c r="AA1" s="38"/>
     </row>
-    <row r="2" spans="1:27" s="21" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:28" s="21" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="14" t="s">
         <v>6</v>
       </c>
@@ -2056,8 +2066,11 @@
       <c r="AA2" s="18" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="3" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB2" s="21" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
       <c r="B3" s="6"/>
       <c r="C3" s="2"/>
@@ -2086,7 +2099,7 @@
       <c r="Z3" s="6"/>
       <c r="AA3" s="5"/>
     </row>
-    <row r="4" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:28" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="6"/>
       <c r="C4" s="2"/>
@@ -2115,7 +2128,7 @@
       <c r="Z4" s="6"/>
       <c r="AA4" s="5"/>
     </row>
-    <row r="5" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:28" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
       <c r="B5" s="6"/>
       <c r="C5" s="2"/>
@@ -2144,7 +2157,7 @@
       <c r="Z5" s="6"/>
       <c r="AA5" s="5"/>
     </row>
-    <row r="6" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:28" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>
       <c r="B6" s="6"/>
       <c r="C6" s="2"/>
@@ -2173,7 +2186,7 @@
       <c r="Z6" s="6"/>
       <c r="AA6" s="5"/>
     </row>
-    <row r="7" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:28" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
       <c r="B7" s="6"/>
       <c r="C7" s="2"/>
@@ -2202,7 +2215,7 @@
       <c r="Z7" s="6"/>
       <c r="AA7" s="5"/>
     </row>
-    <row r="8" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:28" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
       <c r="B8" s="6"/>
       <c r="C8" s="2"/>
@@ -2231,7 +2244,7 @@
       <c r="Z8" s="6"/>
       <c r="AA8" s="5"/>
     </row>
-    <row r="9" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:28" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
       <c r="B9" s="6"/>
       <c r="C9" s="2"/>
@@ -2260,7 +2273,7 @@
       <c r="Z9" s="6"/>
       <c r="AA9" s="5"/>
     </row>
-    <row r="10" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:28" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
       <c r="B10" s="6"/>
       <c r="C10" s="2"/>
@@ -2289,7 +2302,7 @@
       <c r="Z10" s="6"/>
       <c r="AA10" s="5"/>
     </row>
-    <row r="11" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:28" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
         <v>28</v>
       </c>
@@ -2320,7 +2333,7 @@
       <c r="Z11" s="12"/>
       <c r="AA11" s="11"/>
     </row>
-    <row r="12" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="13"/>
       <c r="B12" s="13"/>
       <c r="C12" s="13"/>
@@ -2348,7 +2361,7 @@
       <c r="Y12" s="13"/>
       <c r="Z12" s="19"/>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A13" s="22" t="s">
         <v>29</v>
       </c>
@@ -2379,7 +2392,7 @@
       <c r="Z13" s="24"/>
       <c r="AA13" s="24"/>
     </row>
-    <row r="14" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="13"/>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
@@ -2407,7 +2420,7 @@
       <c r="Y14" s="13"/>
       <c r="Z14" s="19"/>
     </row>
-    <row r="15" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="13"/>
       <c r="B15" s="13"/>
       <c r="C15" s="13"/>
@@ -2435,7 +2448,7 @@
       <c r="Y15" s="13"/>
       <c r="Z15" s="19"/>
     </row>
-    <row r="16" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="13"/>
       <c r="B16" s="13"/>
       <c r="C16" s="13"/>
@@ -29877,12 +29890,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="X1:AA1"/>
     <mergeCell ref="F1:J1"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="K1:O1"/>
     <mergeCell ref="P1:S1"/>
     <mergeCell ref="T1:W1"/>
-    <mergeCell ref="X1:AA1"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>